<commit_message>
Add Control Bucket column and Bucket Details sheet to ruleset template
</commit_message>
<xml_diff>
--- a/backend/templates/sod-sa-analysis/ruleset_template.xlsx
+++ b/backend/templates/sod-sa-analysis/ruleset_template.xlsx
@@ -10,7 +10,8 @@
     <sheet name="SoD Ruleset" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="SA Ruleset" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Entitlement to Privilege" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="How to Fill Data" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Bucket Details" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="How to Fill Data" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -38,23 +39,21 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="14"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00334155"/>
+      <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00334155"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00334155"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -67,17 +66,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F1E3D"/>
+        <fgColor rgb="001F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F7F6F3"/>
+        <fgColor rgb="00375623"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF9E6"/>
+        <fgColor rgb="002E75B6"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,37 +90,43 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="00CCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="00CCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="00CCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00E2E8F0"/>
+        <color rgb="00CCCCCC"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="2"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -489,18 +494,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Control Name</t>
@@ -529,6 +535,11 @@
       <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Risk Description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Control Bucket</t>
         </is>
       </c>
     </row>
@@ -546,15 +557,15 @@
   <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Control Name</t>
@@ -600,12 +611,12 @@
   <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Entitlement Name</t>
@@ -633,388 +644,475 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
-    <col width="82" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1">
+    <row r="1" ht="20" customHeight="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
+          <t>Bucket Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>EY Recommendations</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
           <t>HOW TO FILL DATA — Template Guide</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Overview</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="4" ht="36" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Purpose:</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Defines SOD and SA controls plus the entitlement-to-privilege mapping used to resolve which privileges trigger each control.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Sheets required:</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>All three sheets must be present: 'SoD Ruleset', 'SA Ruleset', 'Entitlement to Privilege'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Three sheets are mandatory: 'SoD Ruleset', 'SA Ruleset', 'Entitlement to Privilege'.  A fourth sheet 'Bucket Details' is optional but required for the Observation tab output.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>SoD Ruleset Sheet</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="8" ht="36" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
         <is>
           <t>Control Name</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Unique SOD control identifier.  Example: 'SOD-001: AP Invoice Creation vs Approval'</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="9" ht="36" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Risk Ranking</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Risk level.  Values: 'High', 'Medium', 'Low'.  Optional — blank → filled with 'Not Provided in SOD SA Ruleset'.</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>LHS Entitlement</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Left-hand-side entitlement of the conflict.  Example: 'Manage Payables Invoices'</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>RHS Entitlement</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Right-hand-side entitlement — must differ from LHS.  Example: 'Approve Payables Invoices'</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
         <is>
           <t>Module(s)</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Oracle module(s) this control covers.  Example: 'Payables'.  Optional.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="13" ht="36" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Risk Description</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>Risk narrative.  Optional — blank → filled with placeholder.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>SA Ruleset Sheet</t>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Control Bucket</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>Groups this SOD control into a named bucket for the Observation tab.  Example: 'Procure to Pay', 'Order to Cash'.  Optional — blank or absent → auto-assigned to 'UNCATEGORIZED'.  Must match a Bucket Name in the Bucket Details sheet for full observation narrative.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
+          <t>SA Ruleset Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="36" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
           <t>Control Name</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Unique SA control identifier.  Example: 'SA-001: System Administration'</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18" ht="36" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Risk Ranking</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Risk level.  Same values as SoD Ruleset.  Optional.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Entitlement</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>The sensitive entitlement.  Example: 'Manage Users'</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="20" ht="36" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Side</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>Side designation.  Typically 'SINGLE' for SA controls.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="21" ht="36" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Module(s)</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>Oracle module(s).  Optional.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Risk Description</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>Risk narrative.  Optional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="22" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Entitlement to Privilege Sheet</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
+          <t>Entitlement to Privilege Sheet</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
           <t>Entitlement Name</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B25" s="6" t="inlineStr">
         <is>
           <t>Must exactly match entitlement names used in SoD Ruleset / SA Ruleset.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Privilege Name</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Display name of the privilege within this entitlement.  Example: 'Manage Payables Invoices'</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Privilege Code</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B27" s="6" t="inlineStr">
         <is>
           <t>System code for the privilege.  Example: 'AP_MANAGE_PAYABLES_INVOICES_PRIV'</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="22" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>Rules &amp; Validation</t>
-        </is>
-      </c>
-    </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Sheet names:</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Must be exactly 'SoD Ruleset', 'SA Ruleset', 'Entitlement to Privilege' — case-sensitive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Critical columns:</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Control Name (both rulesets), LHS/RHS Entitlement (SoD), Entitlement (SA), Entitlement Name + Privilege Code (mapping) — all must be non-empty.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Optional columns:</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>Risk Ranking, Module(s), Risk Description — blanks auto-filled with placeholder.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="22" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>Do's and Don'ts</t>
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Bucket Details Sheet (Optional)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Bucket Name</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Unique name for this bucket.  Must exactly match the Control Bucket values used in the SoD Ruleset sheet.  Example: 'Procure to Pay'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>Narrative describing the risk category for this bucket.  Appears in the Observation tab of the exported Excel report.  Example: 'Unauthorized payments and financial statement manipulation.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>EY Recommendations</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>EY advisory text for this bucket.  Appears in the Observation tab alongside the role count.  Example: 'Implement segregation of duties controls and periodic access reviews.'</t>
         </is>
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="4" t="inlineStr">
         <is>
+          <t>Rules &amp; Validation</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="36" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>Sheet names:</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>Must be exactly 'SoD Ruleset', 'SA Ruleset', 'Entitlement to Privilege' — case-sensitive.  'Bucket Details' is optional.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="36" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>Critical columns:</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>Control Name (both rulesets), LHS/RHS Entitlement (SoD), Entitlement (SA), Entitlement Name + Privilege Code (mapping) — all must be non-empty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="36" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>Optional columns:</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>Risk Ranking, Module(s), Risk Description, Control Bucket, and all Bucket Details columns — blanks are auto-filled with placeholders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="36" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>Control Bucket:</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Ignored at run time if the Observation option is not selected.  Safe to leave blank if the Observation tab is not needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Do's and Don'ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="36" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
           <t>DO:</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B41" s="6" t="inlineStr">
         <is>
           <t>Ensure Entitlement Names in ruleset sheets exactly match the Entitlement Name column in the mapping sheet.</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="42" ht="36" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>DO:</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B42" s="6" t="inlineStr">
         <is>
           <t>Keep Control Names unique within each ruleset sheet.</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="43" ht="36" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>DO:</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>Keep Bucket Names unique in Bucket Details and consistent with Control Bucket values in SoD Ruleset.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="36" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>DON'T:</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B44" s="6" t="inlineStr">
         <is>
           <t>Duplicate Control Names in the same sheet — this causes double-counting.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="45" ht="36" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>DON'T:</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>Add extra sheets — only the three named sheets are read.</t>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>Add extra sheets — only the four named sheets are read.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="31">
-    <mergeCell ref="B17:G17"/>
-    <mergeCell ref="B8:G8"/>
-    <mergeCell ref="B13:G13"/>
-    <mergeCell ref="B29:G29"/>
-    <mergeCell ref="A28:G28"/>
-    <mergeCell ref="B19:G19"/>
-    <mergeCell ref="B34:G34"/>
-    <mergeCell ref="B10:G10"/>
-    <mergeCell ref="B37:G37"/>
-    <mergeCell ref="B9:G9"/>
-    <mergeCell ref="A15:G15"/>
-    <mergeCell ref="B30:G30"/>
-    <mergeCell ref="B24:G24"/>
-    <mergeCell ref="B20:G20"/>
-    <mergeCell ref="A1:G1"/>
-    <mergeCell ref="B5:G5"/>
-    <mergeCell ref="B36:G36"/>
-    <mergeCell ref="B35:G35"/>
-    <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B26:G26"/>
-    <mergeCell ref="A7:G7"/>
-    <mergeCell ref="B25:G25"/>
-    <mergeCell ref="B16:G16"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="B31:G31"/>
-    <mergeCell ref="B12:G12"/>
-    <mergeCell ref="B18:G18"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="B11:G11"/>
-    <mergeCell ref="A23:G23"/>
+  <mergeCells count="8">
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A34:B34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>